<commit_message>
27/10 · Agregar contratista: cantidad de pagos (informes) obligatoria y un solo mensaje al crearlo
- Campo "Cantidad de pagos (informes)" (1 a 24) en Agregar; viaja al CORE (TOTAL INFORMES PRIMARIO)
- El alta pide soloFila: la fila nueva se parcha en memoria (la respuesta pasa de 105 KB a <1 KB)
- El aviso del contrato nuevo sale de fondo (altaAvisos) despues de responder
- Textos: contrasena inicial = documento, un solo mensaje
- Carga masiva: columna opcional PAGOS (INFORMES) en la plantilla y su lectura
- version 2026.10.27.8

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173THzPbnySdMTDTeo8WAQh
</commit_message>
<xml_diff>
--- a/plantillas/PLANTILLA_CARGA_MASIVA_CONTRATISTAS.xlsx
+++ b/plantillas/PLANTILLA_CARGA_MASIVA_CONTRATISTAS.xlsx
@@ -135,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -176,6 +176,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -691,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C31"/>
+  <dimension ref="A2:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -769,7 +772,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Solo se registran las filas que pasaron. Con la casilla de avisos marcada, a cada contratista le llega el aviso (y su contraseña si es nuevo). Sin marcar, se registra en silencio.</t>
+          <t>Solo se registran las filas que pasaron. Con la casilla de avisos marcada, a cada contratista le llega UN mensaje con el aviso del contrato y su acceso (si es nuevo, su contraseña inicial es su cédula). Sin marcar, se registra en silencio.</t>
         </is>
       </c>
     </row>
@@ -925,7 +928,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>10 dígitos, empieza por 3. Ahí le llega su contraseña si es nuevo.</t>
+          <t>10 dígitos, empieza por 3. Ahí le llega el aviso del contrato. Si es nuevo, su contraseña inicial es su número de cédula (con o sin celular).</t>
         </is>
       </c>
     </row>
@@ -953,32 +956,47 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="8" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>PAGOS (INFORMES)</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Opcional, de 1 a 24: los informes o pagos que fija el clausulado. Si la llenas, el contratista ve "1 de N" desde su primer informe y no tiene que escribirlo; si la dejas vacía, él lo escribe en su primer borrador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Leyenda</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>Celda amarilla = se llena. El resto no se toca (no cambies los títulos de la fila 3: la app los reconoce por su nombre).</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="B29" s="8" t="inlineStr">
+    <row r="29" ht="30" customHeight="1"/>
+    <row r="30">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Las mismas reglas del alta de uno</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
+      <c r="C30" s="10" t="inlineStr">
         <is>
           <t>El CORE vuelve a validar todo contra la hoja real antes de registrar: documento, N° de contrato que no exista, fecha de la vigencia, valor, CDP sin usar, secretaría, supervisor con grupo y al menos una obligación.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="11" t="inlineStr">
+    <row r="31"/>
+    <row r="32">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Oscar Polania · Experto en soluciones digitales</t>
         </is>
@@ -995,7 +1013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M303"/>
+  <dimension ref="A1:N303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1011,6 +1029,7 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
     <col width="80" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1091,6 +1110,11 @@
       <c r="M3" s="14" t="inlineStr">
         <is>
           <t>OBLIGACIONES</t>
+        </is>
+      </c>
+      <c r="N3" s="14" t="inlineStr">
+        <is>
+          <t>PAGOS (INFORMES)</t>
         </is>
       </c>
     </row>
@@ -1108,6 +1132,7 @@
       <c r="K4" s="15" t="n"/>
       <c r="L4" s="17" t="n"/>
       <c r="M4" s="16" t="n"/>
+      <c r="N4" s="22" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="n"/>
@@ -1123,6 +1148,7 @@
       <c r="K5" s="15" t="n"/>
       <c r="L5" s="17" t="n"/>
       <c r="M5" s="16" t="n"/>
+      <c r="N5" s="22" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -1138,6 +1164,7 @@
       <c r="K6" s="15" t="n"/>
       <c r="L6" s="17" t="n"/>
       <c r="M6" s="16" t="n"/>
+      <c r="N6" s="22" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -1153,6 +1180,7 @@
       <c r="K7" s="15" t="n"/>
       <c r="L7" s="17" t="n"/>
       <c r="M7" s="16" t="n"/>
+      <c r="N7" s="22" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -1168,6 +1196,7 @@
       <c r="K8" s="15" t="n"/>
       <c r="L8" s="17" t="n"/>
       <c r="M8" s="16" t="n"/>
+      <c r="N8" s="22" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -1183,6 +1212,7 @@
       <c r="K9" s="15" t="n"/>
       <c r="L9" s="17" t="n"/>
       <c r="M9" s="16" t="n"/>
+      <c r="N9" s="22" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -1198,6 +1228,7 @@
       <c r="K10" s="15" t="n"/>
       <c r="L10" s="17" t="n"/>
       <c r="M10" s="16" t="n"/>
+      <c r="N10" s="22" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -1213,6 +1244,7 @@
       <c r="K11" s="15" t="n"/>
       <c r="L11" s="17" t="n"/>
       <c r="M11" s="16" t="n"/>
+      <c r="N11" s="22" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -1228,6 +1260,7 @@
       <c r="K12" s="15" t="n"/>
       <c r="L12" s="17" t="n"/>
       <c r="M12" s="16" t="n"/>
+      <c r="N12" s="22" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -1243,6 +1276,7 @@
       <c r="K13" s="15" t="n"/>
       <c r="L13" s="17" t="n"/>
       <c r="M13" s="16" t="n"/>
+      <c r="N13" s="22" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -1258,6 +1292,7 @@
       <c r="K14" s="15" t="n"/>
       <c r="L14" s="17" t="n"/>
       <c r="M14" s="16" t="n"/>
+      <c r="N14" s="22" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -1273,6 +1308,7 @@
       <c r="K15" s="15" t="n"/>
       <c r="L15" s="17" t="n"/>
       <c r="M15" s="16" t="n"/>
+      <c r="N15" s="22" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -1288,6 +1324,7 @@
       <c r="K16" s="15" t="n"/>
       <c r="L16" s="17" t="n"/>
       <c r="M16" s="16" t="n"/>
+      <c r="N16" s="22" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -1303,6 +1340,7 @@
       <c r="K17" s="15" t="n"/>
       <c r="L17" s="17" t="n"/>
       <c r="M17" s="16" t="n"/>
+      <c r="N17" s="22" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -1318,6 +1356,7 @@
       <c r="K18" s="15" t="n"/>
       <c r="L18" s="17" t="n"/>
       <c r="M18" s="16" t="n"/>
+      <c r="N18" s="22" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -1333,6 +1372,7 @@
       <c r="K19" s="15" t="n"/>
       <c r="L19" s="17" t="n"/>
       <c r="M19" s="16" t="n"/>
+      <c r="N19" s="22" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -1348,6 +1388,7 @@
       <c r="K20" s="15" t="n"/>
       <c r="L20" s="17" t="n"/>
       <c r="M20" s="16" t="n"/>
+      <c r="N20" s="22" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -1363,6 +1404,7 @@
       <c r="K21" s="15" t="n"/>
       <c r="L21" s="17" t="n"/>
       <c r="M21" s="16" t="n"/>
+      <c r="N21" s="22" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -1378,6 +1420,7 @@
       <c r="K22" s="15" t="n"/>
       <c r="L22" s="17" t="n"/>
       <c r="M22" s="16" t="n"/>
+      <c r="N22" s="22" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -1393,6 +1436,7 @@
       <c r="K23" s="15" t="n"/>
       <c r="L23" s="17" t="n"/>
       <c r="M23" s="16" t="n"/>
+      <c r="N23" s="22" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -1408,6 +1452,7 @@
       <c r="K24" s="15" t="n"/>
       <c r="L24" s="17" t="n"/>
       <c r="M24" s="16" t="n"/>
+      <c r="N24" s="22" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="15" t="n"/>
@@ -1423,6 +1468,7 @@
       <c r="K25" s="15" t="n"/>
       <c r="L25" s="17" t="n"/>
       <c r="M25" s="16" t="n"/>
+      <c r="N25" s="22" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="15" t="n"/>
@@ -1438,6 +1484,7 @@
       <c r="K26" s="15" t="n"/>
       <c r="L26" s="17" t="n"/>
       <c r="M26" s="16" t="n"/>
+      <c r="N26" s="22" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="15" t="n"/>
@@ -1453,6 +1500,7 @@
       <c r="K27" s="15" t="n"/>
       <c r="L27" s="17" t="n"/>
       <c r="M27" s="16" t="n"/>
+      <c r="N27" s="22" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="15" t="n"/>
@@ -1468,6 +1516,7 @@
       <c r="K28" s="15" t="n"/>
       <c r="L28" s="17" t="n"/>
       <c r="M28" s="16" t="n"/>
+      <c r="N28" s="22" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="15" t="n"/>
@@ -1483,6 +1532,7 @@
       <c r="K29" s="15" t="n"/>
       <c r="L29" s="17" t="n"/>
       <c r="M29" s="16" t="n"/>
+      <c r="N29" s="22" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="15" t="n"/>
@@ -1498,6 +1548,7 @@
       <c r="K30" s="15" t="n"/>
       <c r="L30" s="17" t="n"/>
       <c r="M30" s="16" t="n"/>
+      <c r="N30" s="22" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="15" t="n"/>
@@ -1513,6 +1564,7 @@
       <c r="K31" s="15" t="n"/>
       <c r="L31" s="17" t="n"/>
       <c r="M31" s="16" t="n"/>
+      <c r="N31" s="22" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="15" t="n"/>
@@ -1528,6 +1580,7 @@
       <c r="K32" s="15" t="n"/>
       <c r="L32" s="17" t="n"/>
       <c r="M32" s="16" t="n"/>
+      <c r="N32" s="22" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="15" t="n"/>
@@ -1543,6 +1596,7 @@
       <c r="K33" s="15" t="n"/>
       <c r="L33" s="17" t="n"/>
       <c r="M33" s="16" t="n"/>
+      <c r="N33" s="22" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="15" t="n"/>
@@ -1558,6 +1612,7 @@
       <c r="K34" s="15" t="n"/>
       <c r="L34" s="17" t="n"/>
       <c r="M34" s="16" t="n"/>
+      <c r="N34" s="22" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="15" t="n"/>
@@ -1573,6 +1628,7 @@
       <c r="K35" s="15" t="n"/>
       <c r="L35" s="17" t="n"/>
       <c r="M35" s="16" t="n"/>
+      <c r="N35" s="22" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="15" t="n"/>
@@ -1588,6 +1644,7 @@
       <c r="K36" s="15" t="n"/>
       <c r="L36" s="17" t="n"/>
       <c r="M36" s="16" t="n"/>
+      <c r="N36" s="22" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="15" t="n"/>
@@ -1603,6 +1660,7 @@
       <c r="K37" s="15" t="n"/>
       <c r="L37" s="17" t="n"/>
       <c r="M37" s="16" t="n"/>
+      <c r="N37" s="22" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="15" t="n"/>
@@ -1618,6 +1676,7 @@
       <c r="K38" s="15" t="n"/>
       <c r="L38" s="17" t="n"/>
       <c r="M38" s="16" t="n"/>
+      <c r="N38" s="22" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="15" t="n"/>
@@ -1633,6 +1692,7 @@
       <c r="K39" s="15" t="n"/>
       <c r="L39" s="17" t="n"/>
       <c r="M39" s="16" t="n"/>
+      <c r="N39" s="22" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="15" t="n"/>
@@ -1648,6 +1708,7 @@
       <c r="K40" s="15" t="n"/>
       <c r="L40" s="17" t="n"/>
       <c r="M40" s="16" t="n"/>
+      <c r="N40" s="22" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="15" t="n"/>
@@ -1663,6 +1724,7 @@
       <c r="K41" s="15" t="n"/>
       <c r="L41" s="17" t="n"/>
       <c r="M41" s="16" t="n"/>
+      <c r="N41" s="22" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="15" t="n"/>
@@ -1678,6 +1740,7 @@
       <c r="K42" s="15" t="n"/>
       <c r="L42" s="17" t="n"/>
       <c r="M42" s="16" t="n"/>
+      <c r="N42" s="22" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="15" t="n"/>
@@ -1693,6 +1756,7 @@
       <c r="K43" s="15" t="n"/>
       <c r="L43" s="17" t="n"/>
       <c r="M43" s="16" t="n"/>
+      <c r="N43" s="22" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="15" t="n"/>
@@ -1708,6 +1772,7 @@
       <c r="K44" s="15" t="n"/>
       <c r="L44" s="17" t="n"/>
       <c r="M44" s="16" t="n"/>
+      <c r="N44" s="22" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="15" t="n"/>
@@ -1723,6 +1788,7 @@
       <c r="K45" s="15" t="n"/>
       <c r="L45" s="17" t="n"/>
       <c r="M45" s="16" t="n"/>
+      <c r="N45" s="22" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="15" t="n"/>
@@ -1738,6 +1804,7 @@
       <c r="K46" s="15" t="n"/>
       <c r="L46" s="17" t="n"/>
       <c r="M46" s="16" t="n"/>
+      <c r="N46" s="22" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="15" t="n"/>
@@ -1753,6 +1820,7 @@
       <c r="K47" s="15" t="n"/>
       <c r="L47" s="17" t="n"/>
       <c r="M47" s="16" t="n"/>
+      <c r="N47" s="22" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="15" t="n"/>
@@ -1768,6 +1836,7 @@
       <c r="K48" s="15" t="n"/>
       <c r="L48" s="17" t="n"/>
       <c r="M48" s="16" t="n"/>
+      <c r="N48" s="22" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="15" t="n"/>
@@ -1783,6 +1852,7 @@
       <c r="K49" s="15" t="n"/>
       <c r="L49" s="17" t="n"/>
       <c r="M49" s="16" t="n"/>
+      <c r="N49" s="22" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="15" t="n"/>
@@ -1798,6 +1868,7 @@
       <c r="K50" s="15" t="n"/>
       <c r="L50" s="17" t="n"/>
       <c r="M50" s="16" t="n"/>
+      <c r="N50" s="22" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="15" t="n"/>
@@ -1813,6 +1884,7 @@
       <c r="K51" s="15" t="n"/>
       <c r="L51" s="17" t="n"/>
       <c r="M51" s="16" t="n"/>
+      <c r="N51" s="22" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="15" t="n"/>
@@ -1828,6 +1900,7 @@
       <c r="K52" s="15" t="n"/>
       <c r="L52" s="17" t="n"/>
       <c r="M52" s="16" t="n"/>
+      <c r="N52" s="22" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="15" t="n"/>
@@ -1843,6 +1916,7 @@
       <c r="K53" s="15" t="n"/>
       <c r="L53" s="17" t="n"/>
       <c r="M53" s="16" t="n"/>
+      <c r="N53" s="22" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="15" t="n"/>
@@ -1858,6 +1932,7 @@
       <c r="K54" s="15" t="n"/>
       <c r="L54" s="17" t="n"/>
       <c r="M54" s="16" t="n"/>
+      <c r="N54" s="22" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="15" t="n"/>
@@ -1873,6 +1948,7 @@
       <c r="K55" s="15" t="n"/>
       <c r="L55" s="17" t="n"/>
       <c r="M55" s="16" t="n"/>
+      <c r="N55" s="22" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="15" t="n"/>
@@ -1888,6 +1964,7 @@
       <c r="K56" s="15" t="n"/>
       <c r="L56" s="17" t="n"/>
       <c r="M56" s="16" t="n"/>
+      <c r="N56" s="22" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="15" t="n"/>
@@ -1903,6 +1980,7 @@
       <c r="K57" s="15" t="n"/>
       <c r="L57" s="17" t="n"/>
       <c r="M57" s="16" t="n"/>
+      <c r="N57" s="22" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="15" t="n"/>
@@ -1918,6 +1996,7 @@
       <c r="K58" s="15" t="n"/>
       <c r="L58" s="17" t="n"/>
       <c r="M58" s="16" t="n"/>
+      <c r="N58" s="22" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="15" t="n"/>
@@ -1933,6 +2012,7 @@
       <c r="K59" s="15" t="n"/>
       <c r="L59" s="17" t="n"/>
       <c r="M59" s="16" t="n"/>
+      <c r="N59" s="22" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="15" t="n"/>
@@ -1948,6 +2028,7 @@
       <c r="K60" s="15" t="n"/>
       <c r="L60" s="17" t="n"/>
       <c r="M60" s="16" t="n"/>
+      <c r="N60" s="22" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="15" t="n"/>
@@ -1963,6 +2044,7 @@
       <c r="K61" s="15" t="n"/>
       <c r="L61" s="17" t="n"/>
       <c r="M61" s="16" t="n"/>
+      <c r="N61" s="22" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="15" t="n"/>
@@ -1978,6 +2060,7 @@
       <c r="K62" s="15" t="n"/>
       <c r="L62" s="17" t="n"/>
       <c r="M62" s="16" t="n"/>
+      <c r="N62" s="22" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="15" t="n"/>
@@ -1993,6 +2076,7 @@
       <c r="K63" s="15" t="n"/>
       <c r="L63" s="17" t="n"/>
       <c r="M63" s="16" t="n"/>
+      <c r="N63" s="22" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="15" t="n"/>
@@ -2008,6 +2092,7 @@
       <c r="K64" s="15" t="n"/>
       <c r="L64" s="17" t="n"/>
       <c r="M64" s="16" t="n"/>
+      <c r="N64" s="22" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="15" t="n"/>
@@ -2023,6 +2108,7 @@
       <c r="K65" s="15" t="n"/>
       <c r="L65" s="17" t="n"/>
       <c r="M65" s="16" t="n"/>
+      <c r="N65" s="22" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="15" t="n"/>
@@ -2038,6 +2124,7 @@
       <c r="K66" s="15" t="n"/>
       <c r="L66" s="17" t="n"/>
       <c r="M66" s="16" t="n"/>
+      <c r="N66" s="22" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="15" t="n"/>
@@ -2053,6 +2140,7 @@
       <c r="K67" s="15" t="n"/>
       <c r="L67" s="17" t="n"/>
       <c r="M67" s="16" t="n"/>
+      <c r="N67" s="22" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="15" t="n"/>
@@ -2068,6 +2156,7 @@
       <c r="K68" s="15" t="n"/>
       <c r="L68" s="17" t="n"/>
       <c r="M68" s="16" t="n"/>
+      <c r="N68" s="22" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="15" t="n"/>
@@ -2083,6 +2172,7 @@
       <c r="K69" s="15" t="n"/>
       <c r="L69" s="17" t="n"/>
       <c r="M69" s="16" t="n"/>
+      <c r="N69" s="22" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="15" t="n"/>
@@ -2098,6 +2188,7 @@
       <c r="K70" s="15" t="n"/>
       <c r="L70" s="17" t="n"/>
       <c r="M70" s="16" t="n"/>
+      <c r="N70" s="22" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="15" t="n"/>
@@ -2113,6 +2204,7 @@
       <c r="K71" s="15" t="n"/>
       <c r="L71" s="17" t="n"/>
       <c r="M71" s="16" t="n"/>
+      <c r="N71" s="22" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="15" t="n"/>
@@ -2128,6 +2220,7 @@
       <c r="K72" s="15" t="n"/>
       <c r="L72" s="17" t="n"/>
       <c r="M72" s="16" t="n"/>
+      <c r="N72" s="22" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="15" t="n"/>
@@ -2143,6 +2236,7 @@
       <c r="K73" s="15" t="n"/>
       <c r="L73" s="17" t="n"/>
       <c r="M73" s="16" t="n"/>
+      <c r="N73" s="22" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="15" t="n"/>
@@ -2158,6 +2252,7 @@
       <c r="K74" s="15" t="n"/>
       <c r="L74" s="17" t="n"/>
       <c r="M74" s="16" t="n"/>
+      <c r="N74" s="22" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="15" t="n"/>
@@ -2173,6 +2268,7 @@
       <c r="K75" s="15" t="n"/>
       <c r="L75" s="17" t="n"/>
       <c r="M75" s="16" t="n"/>
+      <c r="N75" s="22" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="15" t="n"/>
@@ -2188,6 +2284,7 @@
       <c r="K76" s="15" t="n"/>
       <c r="L76" s="17" t="n"/>
       <c r="M76" s="16" t="n"/>
+      <c r="N76" s="22" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="15" t="n"/>
@@ -2203,6 +2300,7 @@
       <c r="K77" s="15" t="n"/>
       <c r="L77" s="17" t="n"/>
       <c r="M77" s="16" t="n"/>
+      <c r="N77" s="22" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="15" t="n"/>
@@ -2218,6 +2316,7 @@
       <c r="K78" s="15" t="n"/>
       <c r="L78" s="17" t="n"/>
       <c r="M78" s="16" t="n"/>
+      <c r="N78" s="22" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="15" t="n"/>
@@ -2233,6 +2332,7 @@
       <c r="K79" s="15" t="n"/>
       <c r="L79" s="17" t="n"/>
       <c r="M79" s="16" t="n"/>
+      <c r="N79" s="22" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="15" t="n"/>
@@ -2248,6 +2348,7 @@
       <c r="K80" s="15" t="n"/>
       <c r="L80" s="17" t="n"/>
       <c r="M80" s="16" t="n"/>
+      <c r="N80" s="22" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="15" t="n"/>
@@ -2263,6 +2364,7 @@
       <c r="K81" s="15" t="n"/>
       <c r="L81" s="17" t="n"/>
       <c r="M81" s="16" t="n"/>
+      <c r="N81" s="22" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="15" t="n"/>
@@ -2278,6 +2380,7 @@
       <c r="K82" s="15" t="n"/>
       <c r="L82" s="17" t="n"/>
       <c r="M82" s="16" t="n"/>
+      <c r="N82" s="22" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="15" t="n"/>
@@ -2293,6 +2396,7 @@
       <c r="K83" s="15" t="n"/>
       <c r="L83" s="17" t="n"/>
       <c r="M83" s="16" t="n"/>
+      <c r="N83" s="22" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="15" t="n"/>
@@ -2308,6 +2412,7 @@
       <c r="K84" s="15" t="n"/>
       <c r="L84" s="17" t="n"/>
       <c r="M84" s="16" t="n"/>
+      <c r="N84" s="22" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="15" t="n"/>
@@ -2323,6 +2428,7 @@
       <c r="K85" s="15" t="n"/>
       <c r="L85" s="17" t="n"/>
       <c r="M85" s="16" t="n"/>
+      <c r="N85" s="22" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="15" t="n"/>
@@ -2338,6 +2444,7 @@
       <c r="K86" s="15" t="n"/>
       <c r="L86" s="17" t="n"/>
       <c r="M86" s="16" t="n"/>
+      <c r="N86" s="22" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="15" t="n"/>
@@ -2353,6 +2460,7 @@
       <c r="K87" s="15" t="n"/>
       <c r="L87" s="17" t="n"/>
       <c r="M87" s="16" t="n"/>
+      <c r="N87" s="22" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="15" t="n"/>
@@ -2368,6 +2476,7 @@
       <c r="K88" s="15" t="n"/>
       <c r="L88" s="17" t="n"/>
       <c r="M88" s="16" t="n"/>
+      <c r="N88" s="22" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="15" t="n"/>
@@ -2383,6 +2492,7 @@
       <c r="K89" s="15" t="n"/>
       <c r="L89" s="17" t="n"/>
       <c r="M89" s="16" t="n"/>
+      <c r="N89" s="22" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="15" t="n"/>
@@ -2398,6 +2508,7 @@
       <c r="K90" s="15" t="n"/>
       <c r="L90" s="17" t="n"/>
       <c r="M90" s="16" t="n"/>
+      <c r="N90" s="22" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="15" t="n"/>
@@ -2413,6 +2524,7 @@
       <c r="K91" s="15" t="n"/>
       <c r="L91" s="17" t="n"/>
       <c r="M91" s="16" t="n"/>
+      <c r="N91" s="22" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="15" t="n"/>
@@ -2428,6 +2540,7 @@
       <c r="K92" s="15" t="n"/>
       <c r="L92" s="17" t="n"/>
       <c r="M92" s="16" t="n"/>
+      <c r="N92" s="22" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="15" t="n"/>
@@ -2443,6 +2556,7 @@
       <c r="K93" s="15" t="n"/>
       <c r="L93" s="17" t="n"/>
       <c r="M93" s="16" t="n"/>
+      <c r="N93" s="22" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="15" t="n"/>
@@ -2458,6 +2572,7 @@
       <c r="K94" s="15" t="n"/>
       <c r="L94" s="17" t="n"/>
       <c r="M94" s="16" t="n"/>
+      <c r="N94" s="22" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="15" t="n"/>
@@ -2473,6 +2588,7 @@
       <c r="K95" s="15" t="n"/>
       <c r="L95" s="17" t="n"/>
       <c r="M95" s="16" t="n"/>
+      <c r="N95" s="22" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="15" t="n"/>
@@ -2488,6 +2604,7 @@
       <c r="K96" s="15" t="n"/>
       <c r="L96" s="17" t="n"/>
       <c r="M96" s="16" t="n"/>
+      <c r="N96" s="22" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="15" t="n"/>
@@ -2503,6 +2620,7 @@
       <c r="K97" s="15" t="n"/>
       <c r="L97" s="17" t="n"/>
       <c r="M97" s="16" t="n"/>
+      <c r="N97" s="22" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="15" t="n"/>
@@ -2518,6 +2636,7 @@
       <c r="K98" s="15" t="n"/>
       <c r="L98" s="17" t="n"/>
       <c r="M98" s="16" t="n"/>
+      <c r="N98" s="22" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="15" t="n"/>
@@ -2533,6 +2652,7 @@
       <c r="K99" s="15" t="n"/>
       <c r="L99" s="17" t="n"/>
       <c r="M99" s="16" t="n"/>
+      <c r="N99" s="22" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="15" t="n"/>
@@ -2548,6 +2668,7 @@
       <c r="K100" s="15" t="n"/>
       <c r="L100" s="17" t="n"/>
       <c r="M100" s="16" t="n"/>
+      <c r="N100" s="22" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="15" t="n"/>
@@ -2563,6 +2684,7 @@
       <c r="K101" s="15" t="n"/>
       <c r="L101" s="17" t="n"/>
       <c r="M101" s="16" t="n"/>
+      <c r="N101" s="22" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="15" t="n"/>
@@ -2578,6 +2700,7 @@
       <c r="K102" s="15" t="n"/>
       <c r="L102" s="17" t="n"/>
       <c r="M102" s="16" t="n"/>
+      <c r="N102" s="22" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="15" t="n"/>
@@ -2593,6 +2716,7 @@
       <c r="K103" s="15" t="n"/>
       <c r="L103" s="17" t="n"/>
       <c r="M103" s="16" t="n"/>
+      <c r="N103" s="22" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="15" t="n"/>
@@ -2608,6 +2732,7 @@
       <c r="K104" s="15" t="n"/>
       <c r="L104" s="17" t="n"/>
       <c r="M104" s="16" t="n"/>
+      <c r="N104" s="22" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="15" t="n"/>
@@ -2623,6 +2748,7 @@
       <c r="K105" s="15" t="n"/>
       <c r="L105" s="17" t="n"/>
       <c r="M105" s="16" t="n"/>
+      <c r="N105" s="22" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="15" t="n"/>
@@ -2638,6 +2764,7 @@
       <c r="K106" s="15" t="n"/>
       <c r="L106" s="17" t="n"/>
       <c r="M106" s="16" t="n"/>
+      <c r="N106" s="22" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="15" t="n"/>
@@ -2653,6 +2780,7 @@
       <c r="K107" s="15" t="n"/>
       <c r="L107" s="17" t="n"/>
       <c r="M107" s="16" t="n"/>
+      <c r="N107" s="22" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="15" t="n"/>
@@ -2668,6 +2796,7 @@
       <c r="K108" s="15" t="n"/>
       <c r="L108" s="17" t="n"/>
       <c r="M108" s="16" t="n"/>
+      <c r="N108" s="22" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="15" t="n"/>
@@ -2683,6 +2812,7 @@
       <c r="K109" s="15" t="n"/>
       <c r="L109" s="17" t="n"/>
       <c r="M109" s="16" t="n"/>
+      <c r="N109" s="22" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="15" t="n"/>
@@ -2698,6 +2828,7 @@
       <c r="K110" s="15" t="n"/>
       <c r="L110" s="17" t="n"/>
       <c r="M110" s="16" t="n"/>
+      <c r="N110" s="22" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="15" t="n"/>
@@ -2713,6 +2844,7 @@
       <c r="K111" s="15" t="n"/>
       <c r="L111" s="17" t="n"/>
       <c r="M111" s="16" t="n"/>
+      <c r="N111" s="22" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="15" t="n"/>
@@ -2728,6 +2860,7 @@
       <c r="K112" s="15" t="n"/>
       <c r="L112" s="17" t="n"/>
       <c r="M112" s="16" t="n"/>
+      <c r="N112" s="22" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="15" t="n"/>
@@ -2743,6 +2876,7 @@
       <c r="K113" s="15" t="n"/>
       <c r="L113" s="17" t="n"/>
       <c r="M113" s="16" t="n"/>
+      <c r="N113" s="22" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="15" t="n"/>
@@ -2758,6 +2892,7 @@
       <c r="K114" s="15" t="n"/>
       <c r="L114" s="17" t="n"/>
       <c r="M114" s="16" t="n"/>
+      <c r="N114" s="22" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="15" t="n"/>
@@ -2773,6 +2908,7 @@
       <c r="K115" s="15" t="n"/>
       <c r="L115" s="17" t="n"/>
       <c r="M115" s="16" t="n"/>
+      <c r="N115" s="22" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="15" t="n"/>
@@ -2788,6 +2924,7 @@
       <c r="K116" s="15" t="n"/>
       <c r="L116" s="17" t="n"/>
       <c r="M116" s="16" t="n"/>
+      <c r="N116" s="22" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="15" t="n"/>
@@ -2803,6 +2940,7 @@
       <c r="K117" s="15" t="n"/>
       <c r="L117" s="17" t="n"/>
       <c r="M117" s="16" t="n"/>
+      <c r="N117" s="22" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="15" t="n"/>
@@ -2818,6 +2956,7 @@
       <c r="K118" s="15" t="n"/>
       <c r="L118" s="17" t="n"/>
       <c r="M118" s="16" t="n"/>
+      <c r="N118" s="22" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="15" t="n"/>
@@ -2833,6 +2972,7 @@
       <c r="K119" s="15" t="n"/>
       <c r="L119" s="17" t="n"/>
       <c r="M119" s="16" t="n"/>
+      <c r="N119" s="22" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="15" t="n"/>
@@ -2848,6 +2988,7 @@
       <c r="K120" s="15" t="n"/>
       <c r="L120" s="17" t="n"/>
       <c r="M120" s="16" t="n"/>
+      <c r="N120" s="22" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="15" t="n"/>
@@ -2863,6 +3004,7 @@
       <c r="K121" s="15" t="n"/>
       <c r="L121" s="17" t="n"/>
       <c r="M121" s="16" t="n"/>
+      <c r="N121" s="22" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="15" t="n"/>
@@ -2878,6 +3020,7 @@
       <c r="K122" s="15" t="n"/>
       <c r="L122" s="17" t="n"/>
       <c r="M122" s="16" t="n"/>
+      <c r="N122" s="22" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="15" t="n"/>
@@ -2893,6 +3036,7 @@
       <c r="K123" s="15" t="n"/>
       <c r="L123" s="17" t="n"/>
       <c r="M123" s="16" t="n"/>
+      <c r="N123" s="22" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="15" t="n"/>
@@ -2908,6 +3052,7 @@
       <c r="K124" s="15" t="n"/>
       <c r="L124" s="17" t="n"/>
       <c r="M124" s="16" t="n"/>
+      <c r="N124" s="22" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="15" t="n"/>
@@ -2923,6 +3068,7 @@
       <c r="K125" s="15" t="n"/>
       <c r="L125" s="17" t="n"/>
       <c r="M125" s="16" t="n"/>
+      <c r="N125" s="22" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="15" t="n"/>
@@ -2938,6 +3084,7 @@
       <c r="K126" s="15" t="n"/>
       <c r="L126" s="17" t="n"/>
       <c r="M126" s="16" t="n"/>
+      <c r="N126" s="22" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="15" t="n"/>
@@ -2953,6 +3100,7 @@
       <c r="K127" s="15" t="n"/>
       <c r="L127" s="17" t="n"/>
       <c r="M127" s="16" t="n"/>
+      <c r="N127" s="22" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="15" t="n"/>
@@ -2968,6 +3116,7 @@
       <c r="K128" s="15" t="n"/>
       <c r="L128" s="17" t="n"/>
       <c r="M128" s="16" t="n"/>
+      <c r="N128" s="22" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="15" t="n"/>
@@ -2983,6 +3132,7 @@
       <c r="K129" s="15" t="n"/>
       <c r="L129" s="17" t="n"/>
       <c r="M129" s="16" t="n"/>
+      <c r="N129" s="22" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="15" t="n"/>
@@ -2998,6 +3148,7 @@
       <c r="K130" s="15" t="n"/>
       <c r="L130" s="17" t="n"/>
       <c r="M130" s="16" t="n"/>
+      <c r="N130" s="22" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="15" t="n"/>
@@ -3013,6 +3164,7 @@
       <c r="K131" s="15" t="n"/>
       <c r="L131" s="17" t="n"/>
       <c r="M131" s="16" t="n"/>
+      <c r="N131" s="22" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="15" t="n"/>
@@ -3028,6 +3180,7 @@
       <c r="K132" s="15" t="n"/>
       <c r="L132" s="17" t="n"/>
       <c r="M132" s="16" t="n"/>
+      <c r="N132" s="22" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="15" t="n"/>
@@ -3043,6 +3196,7 @@
       <c r="K133" s="15" t="n"/>
       <c r="L133" s="17" t="n"/>
       <c r="M133" s="16" t="n"/>
+      <c r="N133" s="22" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="15" t="n"/>
@@ -3058,6 +3212,7 @@
       <c r="K134" s="15" t="n"/>
       <c r="L134" s="17" t="n"/>
       <c r="M134" s="16" t="n"/>
+      <c r="N134" s="22" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="15" t="n"/>
@@ -3073,6 +3228,7 @@
       <c r="K135" s="15" t="n"/>
       <c r="L135" s="17" t="n"/>
       <c r="M135" s="16" t="n"/>
+      <c r="N135" s="22" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="15" t="n"/>
@@ -3088,6 +3244,7 @@
       <c r="K136" s="15" t="n"/>
       <c r="L136" s="17" t="n"/>
       <c r="M136" s="16" t="n"/>
+      <c r="N136" s="22" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="15" t="n"/>
@@ -3103,6 +3260,7 @@
       <c r="K137" s="15" t="n"/>
       <c r="L137" s="17" t="n"/>
       <c r="M137" s="16" t="n"/>
+      <c r="N137" s="22" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="15" t="n"/>
@@ -3118,6 +3276,7 @@
       <c r="K138" s="15" t="n"/>
       <c r="L138" s="17" t="n"/>
       <c r="M138" s="16" t="n"/>
+      <c r="N138" s="22" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="15" t="n"/>
@@ -3133,6 +3292,7 @@
       <c r="K139" s="15" t="n"/>
       <c r="L139" s="17" t="n"/>
       <c r="M139" s="16" t="n"/>
+      <c r="N139" s="22" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="15" t="n"/>
@@ -3148,6 +3308,7 @@
       <c r="K140" s="15" t="n"/>
       <c r="L140" s="17" t="n"/>
       <c r="M140" s="16" t="n"/>
+      <c r="N140" s="22" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="15" t="n"/>
@@ -3163,6 +3324,7 @@
       <c r="K141" s="15" t="n"/>
       <c r="L141" s="17" t="n"/>
       <c r="M141" s="16" t="n"/>
+      <c r="N141" s="22" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="15" t="n"/>
@@ -3178,6 +3340,7 @@
       <c r="K142" s="15" t="n"/>
       <c r="L142" s="17" t="n"/>
       <c r="M142" s="16" t="n"/>
+      <c r="N142" s="22" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="15" t="n"/>
@@ -3193,6 +3356,7 @@
       <c r="K143" s="15" t="n"/>
       <c r="L143" s="17" t="n"/>
       <c r="M143" s="16" t="n"/>
+      <c r="N143" s="22" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="15" t="n"/>
@@ -3208,6 +3372,7 @@
       <c r="K144" s="15" t="n"/>
       <c r="L144" s="17" t="n"/>
       <c r="M144" s="16" t="n"/>
+      <c r="N144" s="22" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="15" t="n"/>
@@ -3223,6 +3388,7 @@
       <c r="K145" s="15" t="n"/>
       <c r="L145" s="17" t="n"/>
       <c r="M145" s="16" t="n"/>
+      <c r="N145" s="22" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="15" t="n"/>
@@ -3238,6 +3404,7 @@
       <c r="K146" s="15" t="n"/>
       <c r="L146" s="17" t="n"/>
       <c r="M146" s="16" t="n"/>
+      <c r="N146" s="22" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="15" t="n"/>
@@ -3253,6 +3420,7 @@
       <c r="K147" s="15" t="n"/>
       <c r="L147" s="17" t="n"/>
       <c r="M147" s="16" t="n"/>
+      <c r="N147" s="22" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="15" t="n"/>
@@ -3268,6 +3436,7 @@
       <c r="K148" s="15" t="n"/>
       <c r="L148" s="17" t="n"/>
       <c r="M148" s="16" t="n"/>
+      <c r="N148" s="22" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="15" t="n"/>
@@ -3283,6 +3452,7 @@
       <c r="K149" s="15" t="n"/>
       <c r="L149" s="17" t="n"/>
       <c r="M149" s="16" t="n"/>
+      <c r="N149" s="22" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="15" t="n"/>
@@ -3298,6 +3468,7 @@
       <c r="K150" s="15" t="n"/>
       <c r="L150" s="17" t="n"/>
       <c r="M150" s="16" t="n"/>
+      <c r="N150" s="22" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="15" t="n"/>
@@ -3313,6 +3484,7 @@
       <c r="K151" s="15" t="n"/>
       <c r="L151" s="17" t="n"/>
       <c r="M151" s="16" t="n"/>
+      <c r="N151" s="22" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="15" t="n"/>
@@ -3328,6 +3500,7 @@
       <c r="K152" s="15" t="n"/>
       <c r="L152" s="17" t="n"/>
       <c r="M152" s="16" t="n"/>
+      <c r="N152" s="22" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="15" t="n"/>
@@ -3343,6 +3516,7 @@
       <c r="K153" s="15" t="n"/>
       <c r="L153" s="17" t="n"/>
       <c r="M153" s="16" t="n"/>
+      <c r="N153" s="22" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="15" t="n"/>
@@ -3358,6 +3532,7 @@
       <c r="K154" s="15" t="n"/>
       <c r="L154" s="17" t="n"/>
       <c r="M154" s="16" t="n"/>
+      <c r="N154" s="22" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="15" t="n"/>
@@ -3373,6 +3548,7 @@
       <c r="K155" s="15" t="n"/>
       <c r="L155" s="17" t="n"/>
       <c r="M155" s="16" t="n"/>
+      <c r="N155" s="22" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="15" t="n"/>
@@ -3388,6 +3564,7 @@
       <c r="K156" s="15" t="n"/>
       <c r="L156" s="17" t="n"/>
       <c r="M156" s="16" t="n"/>
+      <c r="N156" s="22" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="15" t="n"/>
@@ -3403,6 +3580,7 @@
       <c r="K157" s="15" t="n"/>
       <c r="L157" s="17" t="n"/>
       <c r="M157" s="16" t="n"/>
+      <c r="N157" s="22" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="15" t="n"/>
@@ -3418,6 +3596,7 @@
       <c r="K158" s="15" t="n"/>
       <c r="L158" s="17" t="n"/>
       <c r="M158" s="16" t="n"/>
+      <c r="N158" s="22" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="15" t="n"/>
@@ -3433,6 +3612,7 @@
       <c r="K159" s="15" t="n"/>
       <c r="L159" s="17" t="n"/>
       <c r="M159" s="16" t="n"/>
+      <c r="N159" s="22" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="15" t="n"/>
@@ -3448,6 +3628,7 @@
       <c r="K160" s="15" t="n"/>
       <c r="L160" s="17" t="n"/>
       <c r="M160" s="16" t="n"/>
+      <c r="N160" s="22" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="15" t="n"/>
@@ -3463,6 +3644,7 @@
       <c r="K161" s="15" t="n"/>
       <c r="L161" s="17" t="n"/>
       <c r="M161" s="16" t="n"/>
+      <c r="N161" s="22" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="15" t="n"/>
@@ -3478,6 +3660,7 @@
       <c r="K162" s="15" t="n"/>
       <c r="L162" s="17" t="n"/>
       <c r="M162" s="16" t="n"/>
+      <c r="N162" s="22" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="15" t="n"/>
@@ -3493,6 +3676,7 @@
       <c r="K163" s="15" t="n"/>
       <c r="L163" s="17" t="n"/>
       <c r="M163" s="16" t="n"/>
+      <c r="N163" s="22" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="15" t="n"/>
@@ -3508,6 +3692,7 @@
       <c r="K164" s="15" t="n"/>
       <c r="L164" s="17" t="n"/>
       <c r="M164" s="16" t="n"/>
+      <c r="N164" s="22" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="15" t="n"/>
@@ -3523,6 +3708,7 @@
       <c r="K165" s="15" t="n"/>
       <c r="L165" s="17" t="n"/>
       <c r="M165" s="16" t="n"/>
+      <c r="N165" s="22" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="15" t="n"/>
@@ -3538,6 +3724,7 @@
       <c r="K166" s="15" t="n"/>
       <c r="L166" s="17" t="n"/>
       <c r="M166" s="16" t="n"/>
+      <c r="N166" s="22" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="15" t="n"/>
@@ -3553,6 +3740,7 @@
       <c r="K167" s="15" t="n"/>
       <c r="L167" s="17" t="n"/>
       <c r="M167" s="16" t="n"/>
+      <c r="N167" s="22" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="15" t="n"/>
@@ -3568,6 +3756,7 @@
       <c r="K168" s="15" t="n"/>
       <c r="L168" s="17" t="n"/>
       <c r="M168" s="16" t="n"/>
+      <c r="N168" s="22" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="15" t="n"/>
@@ -3583,6 +3772,7 @@
       <c r="K169" s="15" t="n"/>
       <c r="L169" s="17" t="n"/>
       <c r="M169" s="16" t="n"/>
+      <c r="N169" s="22" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="15" t="n"/>
@@ -3598,6 +3788,7 @@
       <c r="K170" s="15" t="n"/>
       <c r="L170" s="17" t="n"/>
       <c r="M170" s="16" t="n"/>
+      <c r="N170" s="22" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="15" t="n"/>
@@ -3613,6 +3804,7 @@
       <c r="K171" s="15" t="n"/>
       <c r="L171" s="17" t="n"/>
       <c r="M171" s="16" t="n"/>
+      <c r="N171" s="22" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="15" t="n"/>
@@ -3628,6 +3820,7 @@
       <c r="K172" s="15" t="n"/>
       <c r="L172" s="17" t="n"/>
       <c r="M172" s="16" t="n"/>
+      <c r="N172" s="22" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="15" t="n"/>
@@ -3643,6 +3836,7 @@
       <c r="K173" s="15" t="n"/>
       <c r="L173" s="17" t="n"/>
       <c r="M173" s="16" t="n"/>
+      <c r="N173" s="22" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="15" t="n"/>
@@ -3658,6 +3852,7 @@
       <c r="K174" s="15" t="n"/>
       <c r="L174" s="17" t="n"/>
       <c r="M174" s="16" t="n"/>
+      <c r="N174" s="22" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="15" t="n"/>
@@ -3673,6 +3868,7 @@
       <c r="K175" s="15" t="n"/>
       <c r="L175" s="17" t="n"/>
       <c r="M175" s="16" t="n"/>
+      <c r="N175" s="22" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="15" t="n"/>
@@ -3688,6 +3884,7 @@
       <c r="K176" s="15" t="n"/>
       <c r="L176" s="17" t="n"/>
       <c r="M176" s="16" t="n"/>
+      <c r="N176" s="22" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="15" t="n"/>
@@ -3703,6 +3900,7 @@
       <c r="K177" s="15" t="n"/>
       <c r="L177" s="17" t="n"/>
       <c r="M177" s="16" t="n"/>
+      <c r="N177" s="22" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="15" t="n"/>
@@ -3718,6 +3916,7 @@
       <c r="K178" s="15" t="n"/>
       <c r="L178" s="17" t="n"/>
       <c r="M178" s="16" t="n"/>
+      <c r="N178" s="22" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="15" t="n"/>
@@ -3733,6 +3932,7 @@
       <c r="K179" s="15" t="n"/>
       <c r="L179" s="17" t="n"/>
       <c r="M179" s="16" t="n"/>
+      <c r="N179" s="22" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="15" t="n"/>
@@ -3748,6 +3948,7 @@
       <c r="K180" s="15" t="n"/>
       <c r="L180" s="17" t="n"/>
       <c r="M180" s="16" t="n"/>
+      <c r="N180" s="22" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="15" t="n"/>
@@ -3763,6 +3964,7 @@
       <c r="K181" s="15" t="n"/>
       <c r="L181" s="17" t="n"/>
       <c r="M181" s="16" t="n"/>
+      <c r="N181" s="22" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="15" t="n"/>
@@ -3778,6 +3980,7 @@
       <c r="K182" s="15" t="n"/>
       <c r="L182" s="17" t="n"/>
       <c r="M182" s="16" t="n"/>
+      <c r="N182" s="22" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="15" t="n"/>
@@ -3793,6 +3996,7 @@
       <c r="K183" s="15" t="n"/>
       <c r="L183" s="17" t="n"/>
       <c r="M183" s="16" t="n"/>
+      <c r="N183" s="22" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="15" t="n"/>
@@ -3808,6 +4012,7 @@
       <c r="K184" s="15" t="n"/>
       <c r="L184" s="17" t="n"/>
       <c r="M184" s="16" t="n"/>
+      <c r="N184" s="22" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="15" t="n"/>
@@ -3823,6 +4028,7 @@
       <c r="K185" s="15" t="n"/>
       <c r="L185" s="17" t="n"/>
       <c r="M185" s="16" t="n"/>
+      <c r="N185" s="22" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="15" t="n"/>
@@ -3838,6 +4044,7 @@
       <c r="K186" s="15" t="n"/>
       <c r="L186" s="17" t="n"/>
       <c r="M186" s="16" t="n"/>
+      <c r="N186" s="22" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="15" t="n"/>
@@ -3853,6 +4060,7 @@
       <c r="K187" s="15" t="n"/>
       <c r="L187" s="17" t="n"/>
       <c r="M187" s="16" t="n"/>
+      <c r="N187" s="22" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="15" t="n"/>
@@ -3868,6 +4076,7 @@
       <c r="K188" s="15" t="n"/>
       <c r="L188" s="17" t="n"/>
       <c r="M188" s="16" t="n"/>
+      <c r="N188" s="22" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="15" t="n"/>
@@ -3883,6 +4092,7 @@
       <c r="K189" s="15" t="n"/>
       <c r="L189" s="17" t="n"/>
       <c r="M189" s="16" t="n"/>
+      <c r="N189" s="22" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="15" t="n"/>
@@ -3898,6 +4108,7 @@
       <c r="K190" s="15" t="n"/>
       <c r="L190" s="17" t="n"/>
       <c r="M190" s="16" t="n"/>
+      <c r="N190" s="22" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="15" t="n"/>
@@ -3913,6 +4124,7 @@
       <c r="K191" s="15" t="n"/>
       <c r="L191" s="17" t="n"/>
       <c r="M191" s="16" t="n"/>
+      <c r="N191" s="22" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="15" t="n"/>
@@ -3928,6 +4140,7 @@
       <c r="K192" s="15" t="n"/>
       <c r="L192" s="17" t="n"/>
       <c r="M192" s="16" t="n"/>
+      <c r="N192" s="22" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="15" t="n"/>
@@ -3943,6 +4156,7 @@
       <c r="K193" s="15" t="n"/>
       <c r="L193" s="17" t="n"/>
       <c r="M193" s="16" t="n"/>
+      <c r="N193" s="22" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="15" t="n"/>
@@ -3958,6 +4172,7 @@
       <c r="K194" s="15" t="n"/>
       <c r="L194" s="17" t="n"/>
       <c r="M194" s="16" t="n"/>
+      <c r="N194" s="22" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="15" t="n"/>
@@ -3973,6 +4188,7 @@
       <c r="K195" s="15" t="n"/>
       <c r="L195" s="17" t="n"/>
       <c r="M195" s="16" t="n"/>
+      <c r="N195" s="22" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="15" t="n"/>
@@ -3988,6 +4204,7 @@
       <c r="K196" s="15" t="n"/>
       <c r="L196" s="17" t="n"/>
       <c r="M196" s="16" t="n"/>
+      <c r="N196" s="22" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="15" t="n"/>
@@ -4003,6 +4220,7 @@
       <c r="K197" s="15" t="n"/>
       <c r="L197" s="17" t="n"/>
       <c r="M197" s="16" t="n"/>
+      <c r="N197" s="22" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="15" t="n"/>
@@ -4018,6 +4236,7 @@
       <c r="K198" s="15" t="n"/>
       <c r="L198" s="17" t="n"/>
       <c r="M198" s="16" t="n"/>
+      <c r="N198" s="22" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="15" t="n"/>
@@ -4033,6 +4252,7 @@
       <c r="K199" s="15" t="n"/>
       <c r="L199" s="17" t="n"/>
       <c r="M199" s="16" t="n"/>
+      <c r="N199" s="22" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="15" t="n"/>
@@ -4048,6 +4268,7 @@
       <c r="K200" s="15" t="n"/>
       <c r="L200" s="17" t="n"/>
       <c r="M200" s="16" t="n"/>
+      <c r="N200" s="22" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="15" t="n"/>
@@ -4063,6 +4284,7 @@
       <c r="K201" s="15" t="n"/>
       <c r="L201" s="17" t="n"/>
       <c r="M201" s="16" t="n"/>
+      <c r="N201" s="22" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="15" t="n"/>
@@ -4078,6 +4300,7 @@
       <c r="K202" s="15" t="n"/>
       <c r="L202" s="17" t="n"/>
       <c r="M202" s="16" t="n"/>
+      <c r="N202" s="22" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="15" t="n"/>
@@ -4093,6 +4316,7 @@
       <c r="K203" s="15" t="n"/>
       <c r="L203" s="17" t="n"/>
       <c r="M203" s="16" t="n"/>
+      <c r="N203" s="22" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="15" t="n"/>
@@ -4108,6 +4332,7 @@
       <c r="K204" s="15" t="n"/>
       <c r="L204" s="17" t="n"/>
       <c r="M204" s="16" t="n"/>
+      <c r="N204" s="22" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="15" t="n"/>
@@ -4123,6 +4348,7 @@
       <c r="K205" s="15" t="n"/>
       <c r="L205" s="17" t="n"/>
       <c r="M205" s="16" t="n"/>
+      <c r="N205" s="22" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="15" t="n"/>
@@ -4138,6 +4364,7 @@
       <c r="K206" s="15" t="n"/>
       <c r="L206" s="17" t="n"/>
       <c r="M206" s="16" t="n"/>
+      <c r="N206" s="22" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="15" t="n"/>
@@ -4153,6 +4380,7 @@
       <c r="K207" s="15" t="n"/>
       <c r="L207" s="17" t="n"/>
       <c r="M207" s="16" t="n"/>
+      <c r="N207" s="22" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="15" t="n"/>
@@ -4168,6 +4396,7 @@
       <c r="K208" s="15" t="n"/>
       <c r="L208" s="17" t="n"/>
       <c r="M208" s="16" t="n"/>
+      <c r="N208" s="22" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="15" t="n"/>
@@ -4183,6 +4412,7 @@
       <c r="K209" s="15" t="n"/>
       <c r="L209" s="17" t="n"/>
       <c r="M209" s="16" t="n"/>
+      <c r="N209" s="22" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="15" t="n"/>
@@ -4198,6 +4428,7 @@
       <c r="K210" s="15" t="n"/>
       <c r="L210" s="17" t="n"/>
       <c r="M210" s="16" t="n"/>
+      <c r="N210" s="22" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="15" t="n"/>
@@ -4213,6 +4444,7 @@
       <c r="K211" s="15" t="n"/>
       <c r="L211" s="17" t="n"/>
       <c r="M211" s="16" t="n"/>
+      <c r="N211" s="22" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="15" t="n"/>
@@ -4228,6 +4460,7 @@
       <c r="K212" s="15" t="n"/>
       <c r="L212" s="17" t="n"/>
       <c r="M212" s="16" t="n"/>
+      <c r="N212" s="22" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="15" t="n"/>
@@ -4243,6 +4476,7 @@
       <c r="K213" s="15" t="n"/>
       <c r="L213" s="17" t="n"/>
       <c r="M213" s="16" t="n"/>
+      <c r="N213" s="22" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="15" t="n"/>
@@ -4258,6 +4492,7 @@
       <c r="K214" s="15" t="n"/>
       <c r="L214" s="17" t="n"/>
       <c r="M214" s="16" t="n"/>
+      <c r="N214" s="22" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="15" t="n"/>
@@ -4273,6 +4508,7 @@
       <c r="K215" s="15" t="n"/>
       <c r="L215" s="17" t="n"/>
       <c r="M215" s="16" t="n"/>
+      <c r="N215" s="22" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="15" t="n"/>
@@ -4288,6 +4524,7 @@
       <c r="K216" s="15" t="n"/>
       <c r="L216" s="17" t="n"/>
       <c r="M216" s="16" t="n"/>
+      <c r="N216" s="22" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="15" t="n"/>
@@ -4303,6 +4540,7 @@
       <c r="K217" s="15" t="n"/>
       <c r="L217" s="17" t="n"/>
       <c r="M217" s="16" t="n"/>
+      <c r="N217" s="22" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="15" t="n"/>
@@ -4318,6 +4556,7 @@
       <c r="K218" s="15" t="n"/>
       <c r="L218" s="17" t="n"/>
       <c r="M218" s="16" t="n"/>
+      <c r="N218" s="22" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="15" t="n"/>
@@ -4333,6 +4572,7 @@
       <c r="K219" s="15" t="n"/>
       <c r="L219" s="17" t="n"/>
       <c r="M219" s="16" t="n"/>
+      <c r="N219" s="22" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="15" t="n"/>
@@ -4348,6 +4588,7 @@
       <c r="K220" s="15" t="n"/>
       <c r="L220" s="17" t="n"/>
       <c r="M220" s="16" t="n"/>
+      <c r="N220" s="22" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="15" t="n"/>
@@ -4363,6 +4604,7 @@
       <c r="K221" s="15" t="n"/>
       <c r="L221" s="17" t="n"/>
       <c r="M221" s="16" t="n"/>
+      <c r="N221" s="22" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="15" t="n"/>
@@ -4378,6 +4620,7 @@
       <c r="K222" s="15" t="n"/>
       <c r="L222" s="17" t="n"/>
       <c r="M222" s="16" t="n"/>
+      <c r="N222" s="22" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="15" t="n"/>
@@ -4393,6 +4636,7 @@
       <c r="K223" s="15" t="n"/>
       <c r="L223" s="17" t="n"/>
       <c r="M223" s="16" t="n"/>
+      <c r="N223" s="22" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="15" t="n"/>
@@ -4408,6 +4652,7 @@
       <c r="K224" s="15" t="n"/>
       <c r="L224" s="17" t="n"/>
       <c r="M224" s="16" t="n"/>
+      <c r="N224" s="22" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="15" t="n"/>
@@ -4423,6 +4668,7 @@
       <c r="K225" s="15" t="n"/>
       <c r="L225" s="17" t="n"/>
       <c r="M225" s="16" t="n"/>
+      <c r="N225" s="22" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="15" t="n"/>
@@ -4438,6 +4684,7 @@
       <c r="K226" s="15" t="n"/>
       <c r="L226" s="17" t="n"/>
       <c r="M226" s="16" t="n"/>
+      <c r="N226" s="22" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="15" t="n"/>
@@ -4453,6 +4700,7 @@
       <c r="K227" s="15" t="n"/>
       <c r="L227" s="17" t="n"/>
       <c r="M227" s="16" t="n"/>
+      <c r="N227" s="22" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="15" t="n"/>
@@ -4468,6 +4716,7 @@
       <c r="K228" s="15" t="n"/>
       <c r="L228" s="17" t="n"/>
       <c r="M228" s="16" t="n"/>
+      <c r="N228" s="22" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="15" t="n"/>
@@ -4483,6 +4732,7 @@
       <c r="K229" s="15" t="n"/>
       <c r="L229" s="17" t="n"/>
       <c r="M229" s="16" t="n"/>
+      <c r="N229" s="22" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="15" t="n"/>
@@ -4498,6 +4748,7 @@
       <c r="K230" s="15" t="n"/>
       <c r="L230" s="17" t="n"/>
       <c r="M230" s="16" t="n"/>
+      <c r="N230" s="22" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="15" t="n"/>
@@ -4513,6 +4764,7 @@
       <c r="K231" s="15" t="n"/>
       <c r="L231" s="17" t="n"/>
       <c r="M231" s="16" t="n"/>
+      <c r="N231" s="22" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="15" t="n"/>
@@ -4528,6 +4780,7 @@
       <c r="K232" s="15" t="n"/>
       <c r="L232" s="17" t="n"/>
       <c r="M232" s="16" t="n"/>
+      <c r="N232" s="22" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="15" t="n"/>
@@ -4543,6 +4796,7 @@
       <c r="K233" s="15" t="n"/>
       <c r="L233" s="17" t="n"/>
       <c r="M233" s="16" t="n"/>
+      <c r="N233" s="22" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="15" t="n"/>
@@ -4558,6 +4812,7 @@
       <c r="K234" s="15" t="n"/>
       <c r="L234" s="17" t="n"/>
       <c r="M234" s="16" t="n"/>
+      <c r="N234" s="22" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="15" t="n"/>
@@ -4573,6 +4828,7 @@
       <c r="K235" s="15" t="n"/>
       <c r="L235" s="17" t="n"/>
       <c r="M235" s="16" t="n"/>
+      <c r="N235" s="22" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="15" t="n"/>
@@ -4588,6 +4844,7 @@
       <c r="K236" s="15" t="n"/>
       <c r="L236" s="17" t="n"/>
       <c r="M236" s="16" t="n"/>
+      <c r="N236" s="22" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="15" t="n"/>
@@ -4603,6 +4860,7 @@
       <c r="K237" s="15" t="n"/>
       <c r="L237" s="17" t="n"/>
       <c r="M237" s="16" t="n"/>
+      <c r="N237" s="22" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="15" t="n"/>
@@ -4618,6 +4876,7 @@
       <c r="K238" s="15" t="n"/>
       <c r="L238" s="17" t="n"/>
       <c r="M238" s="16" t="n"/>
+      <c r="N238" s="22" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="15" t="n"/>
@@ -4633,6 +4892,7 @@
       <c r="K239" s="15" t="n"/>
       <c r="L239" s="17" t="n"/>
       <c r="M239" s="16" t="n"/>
+      <c r="N239" s="22" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="15" t="n"/>
@@ -4648,6 +4908,7 @@
       <c r="K240" s="15" t="n"/>
       <c r="L240" s="17" t="n"/>
       <c r="M240" s="16" t="n"/>
+      <c r="N240" s="22" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="15" t="n"/>
@@ -4663,6 +4924,7 @@
       <c r="K241" s="15" t="n"/>
       <c r="L241" s="17" t="n"/>
       <c r="M241" s="16" t="n"/>
+      <c r="N241" s="22" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="15" t="n"/>
@@ -4678,6 +4940,7 @@
       <c r="K242" s="15" t="n"/>
       <c r="L242" s="17" t="n"/>
       <c r="M242" s="16" t="n"/>
+      <c r="N242" s="22" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="15" t="n"/>
@@ -4693,6 +4956,7 @@
       <c r="K243" s="15" t="n"/>
       <c r="L243" s="17" t="n"/>
       <c r="M243" s="16" t="n"/>
+      <c r="N243" s="22" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="15" t="n"/>
@@ -4708,6 +4972,7 @@
       <c r="K244" s="15" t="n"/>
       <c r="L244" s="17" t="n"/>
       <c r="M244" s="16" t="n"/>
+      <c r="N244" s="22" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="15" t="n"/>
@@ -4723,6 +4988,7 @@
       <c r="K245" s="15" t="n"/>
       <c r="L245" s="17" t="n"/>
       <c r="M245" s="16" t="n"/>
+      <c r="N245" s="22" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="15" t="n"/>
@@ -4738,6 +5004,7 @@
       <c r="K246" s="15" t="n"/>
       <c r="L246" s="17" t="n"/>
       <c r="M246" s="16" t="n"/>
+      <c r="N246" s="22" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="15" t="n"/>
@@ -4753,6 +5020,7 @@
       <c r="K247" s="15" t="n"/>
       <c r="L247" s="17" t="n"/>
       <c r="M247" s="16" t="n"/>
+      <c r="N247" s="22" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="15" t="n"/>
@@ -4768,6 +5036,7 @@
       <c r="K248" s="15" t="n"/>
       <c r="L248" s="17" t="n"/>
       <c r="M248" s="16" t="n"/>
+      <c r="N248" s="22" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="15" t="n"/>
@@ -4783,6 +5052,7 @@
       <c r="K249" s="15" t="n"/>
       <c r="L249" s="17" t="n"/>
       <c r="M249" s="16" t="n"/>
+      <c r="N249" s="22" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="15" t="n"/>
@@ -4798,6 +5068,7 @@
       <c r="K250" s="15" t="n"/>
       <c r="L250" s="17" t="n"/>
       <c r="M250" s="16" t="n"/>
+      <c r="N250" s="22" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="15" t="n"/>
@@ -4813,6 +5084,7 @@
       <c r="K251" s="15" t="n"/>
       <c r="L251" s="17" t="n"/>
       <c r="M251" s="16" t="n"/>
+      <c r="N251" s="22" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="15" t="n"/>
@@ -4828,6 +5100,7 @@
       <c r="K252" s="15" t="n"/>
       <c r="L252" s="17" t="n"/>
       <c r="M252" s="16" t="n"/>
+      <c r="N252" s="22" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="15" t="n"/>
@@ -4843,6 +5116,7 @@
       <c r="K253" s="15" t="n"/>
       <c r="L253" s="17" t="n"/>
       <c r="M253" s="16" t="n"/>
+      <c r="N253" s="22" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="15" t="n"/>
@@ -4858,6 +5132,7 @@
       <c r="K254" s="15" t="n"/>
       <c r="L254" s="17" t="n"/>
       <c r="M254" s="16" t="n"/>
+      <c r="N254" s="22" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="15" t="n"/>
@@ -4873,6 +5148,7 @@
       <c r="K255" s="15" t="n"/>
       <c r="L255" s="17" t="n"/>
       <c r="M255" s="16" t="n"/>
+      <c r="N255" s="22" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="15" t="n"/>
@@ -4888,6 +5164,7 @@
       <c r="K256" s="15" t="n"/>
       <c r="L256" s="17" t="n"/>
       <c r="M256" s="16" t="n"/>
+      <c r="N256" s="22" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="15" t="n"/>
@@ -4903,6 +5180,7 @@
       <c r="K257" s="15" t="n"/>
       <c r="L257" s="17" t="n"/>
       <c r="M257" s="16" t="n"/>
+      <c r="N257" s="22" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="15" t="n"/>
@@ -4918,6 +5196,7 @@
       <c r="K258" s="15" t="n"/>
       <c r="L258" s="17" t="n"/>
       <c r="M258" s="16" t="n"/>
+      <c r="N258" s="22" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="15" t="n"/>
@@ -4933,6 +5212,7 @@
       <c r="K259" s="15" t="n"/>
       <c r="L259" s="17" t="n"/>
       <c r="M259" s="16" t="n"/>
+      <c r="N259" s="22" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="15" t="n"/>
@@ -4948,6 +5228,7 @@
       <c r="K260" s="15" t="n"/>
       <c r="L260" s="17" t="n"/>
       <c r="M260" s="16" t="n"/>
+      <c r="N260" s="22" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="15" t="n"/>
@@ -4963,6 +5244,7 @@
       <c r="K261" s="15" t="n"/>
       <c r="L261" s="17" t="n"/>
       <c r="M261" s="16" t="n"/>
+      <c r="N261" s="22" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="15" t="n"/>
@@ -4978,6 +5260,7 @@
       <c r="K262" s="15" t="n"/>
       <c r="L262" s="17" t="n"/>
       <c r="M262" s="16" t="n"/>
+      <c r="N262" s="22" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="15" t="n"/>
@@ -4993,6 +5276,7 @@
       <c r="K263" s="15" t="n"/>
       <c r="L263" s="17" t="n"/>
       <c r="M263" s="16" t="n"/>
+      <c r="N263" s="22" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="15" t="n"/>
@@ -5008,6 +5292,7 @@
       <c r="K264" s="15" t="n"/>
       <c r="L264" s="17" t="n"/>
       <c r="M264" s="16" t="n"/>
+      <c r="N264" s="22" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="15" t="n"/>
@@ -5023,6 +5308,7 @@
       <c r="K265" s="15" t="n"/>
       <c r="L265" s="17" t="n"/>
       <c r="M265" s="16" t="n"/>
+      <c r="N265" s="22" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="15" t="n"/>
@@ -5038,6 +5324,7 @@
       <c r="K266" s="15" t="n"/>
       <c r="L266" s="17" t="n"/>
       <c r="M266" s="16" t="n"/>
+      <c r="N266" s="22" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="15" t="n"/>
@@ -5053,6 +5340,7 @@
       <c r="K267" s="15" t="n"/>
       <c r="L267" s="17" t="n"/>
       <c r="M267" s="16" t="n"/>
+      <c r="N267" s="22" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="15" t="n"/>
@@ -5068,6 +5356,7 @@
       <c r="K268" s="15" t="n"/>
       <c r="L268" s="17" t="n"/>
       <c r="M268" s="16" t="n"/>
+      <c r="N268" s="22" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="15" t="n"/>
@@ -5083,6 +5372,7 @@
       <c r="K269" s="15" t="n"/>
       <c r="L269" s="17" t="n"/>
       <c r="M269" s="16" t="n"/>
+      <c r="N269" s="22" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="15" t="n"/>
@@ -5098,6 +5388,7 @@
       <c r="K270" s="15" t="n"/>
       <c r="L270" s="17" t="n"/>
       <c r="M270" s="16" t="n"/>
+      <c r="N270" s="22" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="15" t="n"/>
@@ -5113,6 +5404,7 @@
       <c r="K271" s="15" t="n"/>
       <c r="L271" s="17" t="n"/>
       <c r="M271" s="16" t="n"/>
+      <c r="N271" s="22" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="15" t="n"/>
@@ -5128,6 +5420,7 @@
       <c r="K272" s="15" t="n"/>
       <c r="L272" s="17" t="n"/>
       <c r="M272" s="16" t="n"/>
+      <c r="N272" s="22" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="15" t="n"/>
@@ -5143,6 +5436,7 @@
       <c r="K273" s="15" t="n"/>
       <c r="L273" s="17" t="n"/>
       <c r="M273" s="16" t="n"/>
+      <c r="N273" s="22" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="15" t="n"/>
@@ -5158,6 +5452,7 @@
       <c r="K274" s="15" t="n"/>
       <c r="L274" s="17" t="n"/>
       <c r="M274" s="16" t="n"/>
+      <c r="N274" s="22" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="15" t="n"/>
@@ -5173,6 +5468,7 @@
       <c r="K275" s="15" t="n"/>
       <c r="L275" s="17" t="n"/>
       <c r="M275" s="16" t="n"/>
+      <c r="N275" s="22" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="15" t="n"/>
@@ -5188,6 +5484,7 @@
       <c r="K276" s="15" t="n"/>
       <c r="L276" s="17" t="n"/>
       <c r="M276" s="16" t="n"/>
+      <c r="N276" s="22" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="15" t="n"/>
@@ -5203,6 +5500,7 @@
       <c r="K277" s="15" t="n"/>
       <c r="L277" s="17" t="n"/>
       <c r="M277" s="16" t="n"/>
+      <c r="N277" s="22" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="15" t="n"/>
@@ -5218,6 +5516,7 @@
       <c r="K278" s="15" t="n"/>
       <c r="L278" s="17" t="n"/>
       <c r="M278" s="16" t="n"/>
+      <c r="N278" s="22" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="15" t="n"/>
@@ -5233,6 +5532,7 @@
       <c r="K279" s="15" t="n"/>
       <c r="L279" s="17" t="n"/>
       <c r="M279" s="16" t="n"/>
+      <c r="N279" s="22" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="15" t="n"/>
@@ -5248,6 +5548,7 @@
       <c r="K280" s="15" t="n"/>
       <c r="L280" s="17" t="n"/>
       <c r="M280" s="16" t="n"/>
+      <c r="N280" s="22" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="15" t="n"/>
@@ -5263,6 +5564,7 @@
       <c r="K281" s="15" t="n"/>
       <c r="L281" s="17" t="n"/>
       <c r="M281" s="16" t="n"/>
+      <c r="N281" s="22" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="15" t="n"/>
@@ -5278,6 +5580,7 @@
       <c r="K282" s="15" t="n"/>
       <c r="L282" s="17" t="n"/>
       <c r="M282" s="16" t="n"/>
+      <c r="N282" s="22" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="15" t="n"/>
@@ -5293,6 +5596,7 @@
       <c r="K283" s="15" t="n"/>
       <c r="L283" s="17" t="n"/>
       <c r="M283" s="16" t="n"/>
+      <c r="N283" s="22" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="15" t="n"/>
@@ -5308,6 +5612,7 @@
       <c r="K284" s="15" t="n"/>
       <c r="L284" s="17" t="n"/>
       <c r="M284" s="16" t="n"/>
+      <c r="N284" s="22" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="15" t="n"/>
@@ -5323,6 +5628,7 @@
       <c r="K285" s="15" t="n"/>
       <c r="L285" s="17" t="n"/>
       <c r="M285" s="16" t="n"/>
+      <c r="N285" s="22" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="15" t="n"/>
@@ -5338,6 +5644,7 @@
       <c r="K286" s="15" t="n"/>
       <c r="L286" s="17" t="n"/>
       <c r="M286" s="16" t="n"/>
+      <c r="N286" s="22" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="15" t="n"/>
@@ -5353,6 +5660,7 @@
       <c r="K287" s="15" t="n"/>
       <c r="L287" s="17" t="n"/>
       <c r="M287" s="16" t="n"/>
+      <c r="N287" s="22" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="15" t="n"/>
@@ -5368,6 +5676,7 @@
       <c r="K288" s="15" t="n"/>
       <c r="L288" s="17" t="n"/>
       <c r="M288" s="16" t="n"/>
+      <c r="N288" s="22" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="15" t="n"/>
@@ -5383,6 +5692,7 @@
       <c r="K289" s="15" t="n"/>
       <c r="L289" s="17" t="n"/>
       <c r="M289" s="16" t="n"/>
+      <c r="N289" s="22" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="15" t="n"/>
@@ -5398,6 +5708,7 @@
       <c r="K290" s="15" t="n"/>
       <c r="L290" s="17" t="n"/>
       <c r="M290" s="16" t="n"/>
+      <c r="N290" s="22" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="15" t="n"/>
@@ -5413,6 +5724,7 @@
       <c r="K291" s="15" t="n"/>
       <c r="L291" s="17" t="n"/>
       <c r="M291" s="16" t="n"/>
+      <c r="N291" s="22" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="15" t="n"/>
@@ -5428,6 +5740,7 @@
       <c r="K292" s="15" t="n"/>
       <c r="L292" s="17" t="n"/>
       <c r="M292" s="16" t="n"/>
+      <c r="N292" s="22" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="15" t="n"/>
@@ -5443,6 +5756,7 @@
       <c r="K293" s="15" t="n"/>
       <c r="L293" s="17" t="n"/>
       <c r="M293" s="16" t="n"/>
+      <c r="N293" s="22" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="15" t="n"/>
@@ -5458,6 +5772,7 @@
       <c r="K294" s="15" t="n"/>
       <c r="L294" s="17" t="n"/>
       <c r="M294" s="16" t="n"/>
+      <c r="N294" s="22" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="15" t="n"/>
@@ -5473,6 +5788,7 @@
       <c r="K295" s="15" t="n"/>
       <c r="L295" s="17" t="n"/>
       <c r="M295" s="16" t="n"/>
+      <c r="N295" s="22" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="15" t="n"/>
@@ -5488,6 +5804,7 @@
       <c r="K296" s="15" t="n"/>
       <c r="L296" s="17" t="n"/>
       <c r="M296" s="16" t="n"/>
+      <c r="N296" s="22" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="15" t="n"/>
@@ -5503,6 +5820,7 @@
       <c r="K297" s="15" t="n"/>
       <c r="L297" s="17" t="n"/>
       <c r="M297" s="16" t="n"/>
+      <c r="N297" s="22" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="15" t="n"/>
@@ -5518,6 +5836,7 @@
       <c r="K298" s="15" t="n"/>
       <c r="L298" s="17" t="n"/>
       <c r="M298" s="16" t="n"/>
+      <c r="N298" s="22" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="15" t="n"/>
@@ -5533,6 +5852,7 @@
       <c r="K299" s="15" t="n"/>
       <c r="L299" s="17" t="n"/>
       <c r="M299" s="16" t="n"/>
+      <c r="N299" s="22" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="15" t="n"/>
@@ -5548,6 +5868,7 @@
       <c r="K300" s="15" t="n"/>
       <c r="L300" s="17" t="n"/>
       <c r="M300" s="16" t="n"/>
+      <c r="N300" s="22" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="15" t="n"/>
@@ -5563,6 +5884,7 @@
       <c r="K301" s="15" t="n"/>
       <c r="L301" s="17" t="n"/>
       <c r="M301" s="16" t="n"/>
+      <c r="N301" s="22" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="15" t="n"/>
@@ -5578,6 +5900,7 @@
       <c r="K302" s="15" t="n"/>
       <c r="L302" s="17" t="n"/>
       <c r="M302" s="16" t="n"/>
+      <c r="N302" s="22" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="15" t="n"/>
@@ -5593,9 +5916,10 @@
       <c r="K303" s="15" t="n"/>
       <c r="L303" s="17" t="n"/>
       <c r="M303" s="16" t="n"/>
+      <c r="N303" s="22" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="8">
     <dataValidation sqref="I4:I303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="No está en la lista" error="Escoge la secretaría de la lista." type="list">
       <formula1>=LISTAS!$A$2:$A$8</formula1>
     </dataValidation>
@@ -5620,6 +5944,10 @@
       <formula1>100000</formula1>
       <formula2>9999999999</formula2>
     </dataValidation>
+    <dataValidation sqref="N4:N303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pagos" error="De 1 a 24: los informes o pagos que fija el clausulado." type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>24</formula2>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5632,7 +5960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5648,6 +5976,7 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
     <col width="80" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5730,6 +6059,11 @@
           <t>OBLIGACIONES</t>
         </is>
       </c>
+      <c r="N3" s="14" t="inlineStr">
+        <is>
+          <t>PAGOS (INFORMES)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="75" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
@@ -5792,6 +6126,9 @@
         <is>
           <t>1. Apoyar la organización del archivo de gestión de la secretaría. 2. Atender y orientar a los usuarios que lleguen a la dependencia. 3. Presentar el informe mensual de actividades con sus evidencias.</t>
         </is>
+      </c>
+      <c r="N4" s="15" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="6">

</xml_diff>